<commit_message>
Normalizer data and performance fix
</commit_message>
<xml_diff>
--- a/sample_data/projectX_Timesheet_December 2024.xlsx
+++ b/sample_data/projectX_Timesheet_December 2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\takumar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snarayanaswamy/Documents/hackaton/finintel_run/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75BDC06-671D-4E79-8922-E634770DF5DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EBE5BB-969E-A24B-9CDE-AEB7264B5CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{D17B7CAD-D25E-4F20-8096-0A9ACC033B04}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" activeTab="1" xr2:uid="{D17B7CAD-D25E-4F20-8096-0A9ACC033B04}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="6" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="135">
   <si>
     <t>Onboard date</t>
   </si>
@@ -447,13 +447,17 @@
   </si>
   <si>
     <t>ProjectX</t>
+  </si>
+  <si>
+    <t>cost_rate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
@@ -674,7 +678,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -730,6 +734,18 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -744,24 +760,32 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="6" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="89">
+  <dxfs count="91">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1532,6 +1556,20 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.59996337778862885"/>
@@ -1583,9 +1621,6 @@
           <bgColor rgb="FFFF0066"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <font>
@@ -2324,6 +2359,9 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <font>
@@ -2373,65 +2411,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{86BD8C17-1601-4130-BC1E-DD75642252C4}" name="Table27" displayName="Table27" ref="E5:AR21" totalsRowCount="1" headerRowDxfId="88" dataDxfId="87">
-  <tableColumns count="40">
-    <tableColumn id="40" xr3:uid="{0A54AE2F-C256-4AA4-81C3-E00ACCC76EC8}" name="Emp ID" dataDxfId="86" totalsRowDxfId="39"/>
-    <tableColumn id="39" xr3:uid="{9669CAB7-33E5-40E8-9ECD-BFA5F383C0BD}" name="Role as per SoW" dataDxfId="85" totalsRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{86BD8C17-1601-4130-BC1E-DD75642252C4}" name="Table27" displayName="Table27" ref="E5:AS21" totalsRowCount="1" headerRowDxfId="90" dataDxfId="89">
+  <tableColumns count="41">
+    <tableColumn id="40" xr3:uid="{0A54AE2F-C256-4AA4-81C3-E00ACCC76EC8}" name="Emp ID" dataDxfId="87" totalsRowDxfId="40"/>
+    <tableColumn id="39" xr3:uid="{9669CAB7-33E5-40E8-9ECD-BFA5F383C0BD}" name="Role as per SoW" dataDxfId="86" totalsRowDxfId="39">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Role as per SoW])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{4449859A-55A6-45AA-8A96-FCC6309D5F60}" name="Name" totalsRowLabel="Total" dataDxfId="84" totalsRowDxfId="37">
+    <tableColumn id="1" xr3:uid="{4449859A-55A6-45AA-8A96-FCC6309D5F60}" name="Name" totalsRowLabel="Total" dataDxfId="85" totalsRowDxfId="38">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Name])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{25895A40-683C-400E-B977-6736C26F70FF}" name="Max Billable Hours" totalsRowFunction="sum" dataDxfId="83" totalsRowDxfId="36">
+    <tableColumn id="2" xr3:uid="{25895A40-683C-400E-B977-6736C26F70FF}" name="Max Billable Hours" totalsRowFunction="sum" dataDxfId="84" totalsRowDxfId="37">
       <calculatedColumnFormula>IF(Table27[[#This Row],[Status]]="Active",SUM(COUNT(Table27[[#This Row],[1]:[31]]), COUNTIF(Table27[[#This Row],[1]:[31]],"OFF"))*_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Billable Hours per day]),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{42257E96-50F7-4B29-B3B1-132233AB2AA6}" name="Actual Hours" totalsRowFunction="sum" dataDxfId="82" totalsRowDxfId="35">
+    <tableColumn id="3" xr3:uid="{42257E96-50F7-4B29-B3B1-132233AB2AA6}" name="Actual Hours" totalsRowFunction="sum" dataDxfId="83" totalsRowDxfId="36">
       <calculatedColumnFormula>IF(Table27[[#This Row],[Status]]="Active",SUM(Table27[[#This Row],[1]:[31]]),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{C4F1F072-CB0B-4451-B5C6-05FB81DFFC03}" name="Rate" dataDxfId="81" totalsRowDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{6E3636B9-97B1-4231-848A-84020E8CD1A3}" name="Final Billing Amount" totalsRowFunction="sum" dataDxfId="80" totalsRowDxfId="33">
+    <tableColumn id="4" xr3:uid="{C4F1F072-CB0B-4451-B5C6-05FB81DFFC03}" name="Rate" dataDxfId="82" totalsRowDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{6E3636B9-97B1-4231-848A-84020E8CD1A3}" name="Final Billing Amount" totalsRowFunction="sum" dataDxfId="81" totalsRowDxfId="34">
       <calculatedColumnFormula>IFERROR(Table27[[#This Row],[Actual Hours]]*Table27[[#This Row],[Rate]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{D4793879-E2F3-472D-8E9B-2105426B8F6B}" name="1" totalsRowFunction="sum" dataDxfId="79" totalsRowDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{E486E4A8-41C0-4AFF-BB9A-B45102FE633C}" name="2" totalsRowFunction="sum" dataDxfId="78" totalsRowDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{4A4F0742-3816-4B9E-9F0A-7F96C051FEC1}" name="3" totalsRowFunction="sum" dataDxfId="77" totalsRowDxfId="30"/>
-    <tableColumn id="9" xr3:uid="{24E6AAA5-D211-40AD-808B-294BCA6071A0}" name="4" totalsRowFunction="sum" dataDxfId="76" totalsRowDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{70086128-55FD-4B5D-AE29-F9B280C62589}" name="5" totalsRowFunction="sum" dataDxfId="75" totalsRowDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{F86580CD-5B8C-4123-A821-D46F4A6EC4F6}" name="6" totalsRowFunction="sum" dataDxfId="74" totalsRowDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{6F961A6F-63D3-4D42-AE89-E86613A2C14F}" name="7" totalsRowFunction="sum" dataDxfId="73" totalsRowDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{554D2725-AA19-4B75-A7B9-2A8387E18BDC}" name="8" totalsRowFunction="sum" dataDxfId="72" totalsRowDxfId="25"/>
-    <tableColumn id="14" xr3:uid="{63D8B858-12A3-4A0B-A826-BE3186D9F21F}" name="9" totalsRowFunction="sum" dataDxfId="71" totalsRowDxfId="24"/>
-    <tableColumn id="15" xr3:uid="{B19FFC3C-59E3-475E-8113-0CE80BFE9635}" name="10" totalsRowFunction="sum" dataDxfId="70" totalsRowDxfId="23"/>
-    <tableColumn id="16" xr3:uid="{D5D68AE4-2278-40D7-BFED-A0B492731248}" name="11" totalsRowFunction="sum" dataDxfId="69" totalsRowDxfId="22"/>
-    <tableColumn id="17" xr3:uid="{30651372-2451-4B32-ACB6-665FBA20F98B}" name="12" totalsRowFunction="sum" dataDxfId="68" totalsRowDxfId="21"/>
-    <tableColumn id="18" xr3:uid="{D0FAAF2E-7D84-4E6B-90D7-80E1E12AFF8B}" name="13" totalsRowFunction="sum" dataDxfId="67" totalsRowDxfId="20"/>
-    <tableColumn id="19" xr3:uid="{DA2E8EE3-9D9F-4FCB-B634-0F5CDF5A99C6}" name="14" totalsRowFunction="sum" dataDxfId="66" totalsRowDxfId="19"/>
-    <tableColumn id="20" xr3:uid="{27F58B70-B194-47CB-B393-AB8FB149C0CD}" name="15" totalsRowFunction="sum" dataDxfId="65" totalsRowDxfId="18"/>
-    <tableColumn id="21" xr3:uid="{A626272B-9B6C-49DD-B884-912D4983CB24}" name="16" totalsRowFunction="sum" dataDxfId="64" totalsRowDxfId="17"/>
-    <tableColumn id="22" xr3:uid="{2D327AA4-6E26-4B2B-A188-C61BB78F1A4F}" name="17" totalsRowFunction="sum" dataDxfId="63" totalsRowDxfId="16"/>
-    <tableColumn id="23" xr3:uid="{81418BDA-3722-4FD6-A1AC-D19EC0365795}" name="18" totalsRowFunction="sum" dataDxfId="62" totalsRowDxfId="15"/>
-    <tableColumn id="24" xr3:uid="{748261B7-3B42-48B0-B56D-6066930E4F45}" name="19" totalsRowFunction="sum" dataDxfId="61" totalsRowDxfId="14"/>
-    <tableColumn id="25" xr3:uid="{27D1FC17-EEA9-4BBA-9BF0-F488BB07BC27}" name="20" totalsRowFunction="sum" dataDxfId="60" totalsRowDxfId="13"/>
-    <tableColumn id="26" xr3:uid="{CE5F7E04-EA29-476A-8C04-10311E5AA245}" name="21" totalsRowFunction="sum" dataDxfId="59" totalsRowDxfId="12"/>
-    <tableColumn id="27" xr3:uid="{6A1ED293-6B3A-4F5F-878E-BC6852209689}" name="22" totalsRowFunction="sum" dataDxfId="58" totalsRowDxfId="11"/>
-    <tableColumn id="28" xr3:uid="{DED4194D-2CE9-4CED-A0E1-5517221173CE}" name="23" totalsRowFunction="sum" dataDxfId="57" totalsRowDxfId="10"/>
-    <tableColumn id="29" xr3:uid="{8F702A72-079F-4DDC-8889-42FF1892A8D9}" name="24" totalsRowFunction="sum" dataDxfId="56" totalsRowDxfId="9"/>
-    <tableColumn id="30" xr3:uid="{952EC144-0583-4A0E-9606-7D1C67415A11}" name="25" totalsRowFunction="sum" dataDxfId="55" totalsRowDxfId="8"/>
-    <tableColumn id="31" xr3:uid="{02E5AB35-203D-45F7-968D-89FFFD7605BD}" name="26" totalsRowFunction="sum" dataDxfId="54" totalsRowDxfId="7"/>
-    <tableColumn id="32" xr3:uid="{74C12FEA-BDE5-479D-93E6-E783309D1823}" name="27" totalsRowFunction="sum" dataDxfId="53" totalsRowDxfId="6"/>
-    <tableColumn id="33" xr3:uid="{9340BC5C-0231-47F4-BAAB-F3EC43CAB876}" name="28" totalsRowFunction="sum" dataDxfId="52" totalsRowDxfId="5"/>
-    <tableColumn id="34" xr3:uid="{3EAF38D2-F687-4B74-91B5-FCEBE8F0AF14}" name="29" totalsRowFunction="sum" dataDxfId="51" totalsRowDxfId="4"/>
-    <tableColumn id="35" xr3:uid="{EA5A44B8-FFE4-4939-963A-C719186ADF9D}" name="30" totalsRowFunction="sum" dataDxfId="50" totalsRowDxfId="3"/>
-    <tableColumn id="36" xr3:uid="{F4FC74EA-7D3E-4BCD-81C3-3AD31C403124}" name="31" totalsRowFunction="custom" dataDxfId="49" totalsRowDxfId="2">
+    <tableColumn id="6" xr3:uid="{D4793879-E2F3-472D-8E9B-2105426B8F6B}" name="1" totalsRowFunction="sum" dataDxfId="80" totalsRowDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{E486E4A8-41C0-4AFF-BB9A-B45102FE633C}" name="2" totalsRowFunction="sum" dataDxfId="79" totalsRowDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{4A4F0742-3816-4B9E-9F0A-7F96C051FEC1}" name="3" totalsRowFunction="sum" dataDxfId="78" totalsRowDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{24E6AAA5-D211-40AD-808B-294BCA6071A0}" name="4" totalsRowFunction="sum" dataDxfId="77" totalsRowDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{70086128-55FD-4B5D-AE29-F9B280C62589}" name="5" totalsRowFunction="sum" dataDxfId="76" totalsRowDxfId="29"/>
+    <tableColumn id="11" xr3:uid="{F86580CD-5B8C-4123-A821-D46F4A6EC4F6}" name="6" totalsRowFunction="sum" dataDxfId="75" totalsRowDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{6F961A6F-63D3-4D42-AE89-E86613A2C14F}" name="7" totalsRowFunction="sum" dataDxfId="74" totalsRowDxfId="27"/>
+    <tableColumn id="13" xr3:uid="{554D2725-AA19-4B75-A7B9-2A8387E18BDC}" name="8" totalsRowFunction="sum" dataDxfId="73" totalsRowDxfId="26"/>
+    <tableColumn id="14" xr3:uid="{63D8B858-12A3-4A0B-A826-BE3186D9F21F}" name="9" totalsRowFunction="sum" dataDxfId="72" totalsRowDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{B19FFC3C-59E3-475E-8113-0CE80BFE9635}" name="10" totalsRowFunction="sum" dataDxfId="71" totalsRowDxfId="24"/>
+    <tableColumn id="16" xr3:uid="{D5D68AE4-2278-40D7-BFED-A0B492731248}" name="11" totalsRowFunction="sum" dataDxfId="70" totalsRowDxfId="23"/>
+    <tableColumn id="17" xr3:uid="{30651372-2451-4B32-ACB6-665FBA20F98B}" name="12" totalsRowFunction="sum" dataDxfId="69" totalsRowDxfId="22"/>
+    <tableColumn id="18" xr3:uid="{D0FAAF2E-7D84-4E6B-90D7-80E1E12AFF8B}" name="13" totalsRowFunction="sum" dataDxfId="68" totalsRowDxfId="21"/>
+    <tableColumn id="19" xr3:uid="{DA2E8EE3-9D9F-4FCB-B634-0F5CDF5A99C6}" name="14" totalsRowFunction="sum" dataDxfId="67" totalsRowDxfId="20"/>
+    <tableColumn id="20" xr3:uid="{27F58B70-B194-47CB-B393-AB8FB149C0CD}" name="15" totalsRowFunction="sum" dataDxfId="66" totalsRowDxfId="19"/>
+    <tableColumn id="21" xr3:uid="{A626272B-9B6C-49DD-B884-912D4983CB24}" name="16" totalsRowFunction="sum" dataDxfId="65" totalsRowDxfId="18"/>
+    <tableColumn id="22" xr3:uid="{2D327AA4-6E26-4B2B-A188-C61BB78F1A4F}" name="17" totalsRowFunction="sum" dataDxfId="64" totalsRowDxfId="17"/>
+    <tableColumn id="23" xr3:uid="{81418BDA-3722-4FD6-A1AC-D19EC0365795}" name="18" totalsRowFunction="sum" dataDxfId="63" totalsRowDxfId="16"/>
+    <tableColumn id="24" xr3:uid="{748261B7-3B42-48B0-B56D-6066930E4F45}" name="19" totalsRowFunction="sum" dataDxfId="62" totalsRowDxfId="15"/>
+    <tableColumn id="25" xr3:uid="{27D1FC17-EEA9-4BBA-9BF0-F488BB07BC27}" name="20" totalsRowFunction="sum" dataDxfId="61" totalsRowDxfId="14"/>
+    <tableColumn id="26" xr3:uid="{CE5F7E04-EA29-476A-8C04-10311E5AA245}" name="21" totalsRowFunction="sum" dataDxfId="60" totalsRowDxfId="13"/>
+    <tableColumn id="27" xr3:uid="{6A1ED293-6B3A-4F5F-878E-BC6852209689}" name="22" totalsRowFunction="sum" dataDxfId="59" totalsRowDxfId="12"/>
+    <tableColumn id="28" xr3:uid="{DED4194D-2CE9-4CED-A0E1-5517221173CE}" name="23" totalsRowFunction="sum" dataDxfId="58" totalsRowDxfId="11"/>
+    <tableColumn id="29" xr3:uid="{8F702A72-079F-4DDC-8889-42FF1892A8D9}" name="24" totalsRowFunction="sum" dataDxfId="57" totalsRowDxfId="10"/>
+    <tableColumn id="30" xr3:uid="{952EC144-0583-4A0E-9606-7D1C67415A11}" name="25" totalsRowFunction="sum" dataDxfId="56" totalsRowDxfId="9"/>
+    <tableColumn id="31" xr3:uid="{02E5AB35-203D-45F7-968D-89FFFD7605BD}" name="26" totalsRowFunction="sum" dataDxfId="55" totalsRowDxfId="8"/>
+    <tableColumn id="32" xr3:uid="{74C12FEA-BDE5-479D-93E6-E783309D1823}" name="27" totalsRowFunction="sum" dataDxfId="54" totalsRowDxfId="7"/>
+    <tableColumn id="33" xr3:uid="{9340BC5C-0231-47F4-BAAB-F3EC43CAB876}" name="28" totalsRowFunction="sum" dataDxfId="53" totalsRowDxfId="6"/>
+    <tableColumn id="34" xr3:uid="{3EAF38D2-F687-4B74-91B5-FCEBE8F0AF14}" name="29" totalsRowFunction="sum" dataDxfId="52" totalsRowDxfId="5"/>
+    <tableColumn id="35" xr3:uid="{EA5A44B8-FFE4-4939-963A-C719186ADF9D}" name="30" totalsRowFunction="sum" dataDxfId="51" totalsRowDxfId="4"/>
+    <tableColumn id="36" xr3:uid="{F4FC74EA-7D3E-4BCD-81C3-3AD31C403124}" name="31" totalsRowFunction="custom" dataDxfId="50" totalsRowDxfId="3">
       <totalsRowFormula>SUBTOTAL(109,Table27[30])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="38" xr3:uid="{04D5C202-3AEB-4435-9159-2F359239778C}" name="Status" dataDxfId="48" totalsRowDxfId="1">
+    <tableColumn id="38" xr3:uid="{04D5C202-3AEB-4435-9159-2F359239778C}" name="Status" dataDxfId="49" totalsRowDxfId="2">
       <calculatedColumnFormula>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="37" xr3:uid="{CF7A8946-2CDE-4C23-8580-6C1FEFBCBE31}" name="Billing %" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="0">
+    <tableColumn id="37" xr3:uid="{CF7A8946-2CDE-4C23-8580-6C1FEFBCBE31}" name="Billing %" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="1">
       <calculatedColumnFormula>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</calculatedColumnFormula>
       <totalsRowFormula>Table27[[#Totals],[Actual Hours]]/Table27[[#Totals],[Max Billable Hours]]</totalsRowFormula>
     </tableColumn>
+    <tableColumn id="43" xr3:uid="{BA0B4D40-6A92-BC4F-88CE-8065716F8E76}" name="cost_rate" dataDxfId="41" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
 </table>
@@ -2444,7 +2483,7 @@
     <tableColumn id="7" xr3:uid="{B318C1B5-DDBA-40C0-AEBF-DD0C8A713529}" name="Emp ID"/>
     <tableColumn id="1" xr3:uid="{61F66100-680B-43D4-9643-C6580DB98E19}" name="Name"/>
     <tableColumn id="2" xr3:uid="{1F30959A-FED7-4B38-99D5-577C9DC6ADAE}" name="Role as per SoW"/>
-    <tableColumn id="3" xr3:uid="{A55B2A4F-0240-4914-A04B-C9F5FB352057}" name="Onboard date" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{A55B2A4F-0240-4914-A04B-C9F5FB352057}" name="Onboard date" dataDxfId="88"/>
     <tableColumn id="4" xr3:uid="{339185EB-1D1C-416C-A786-1371EE5CAED8}" name="Status"/>
     <tableColumn id="5" xr3:uid="{FD8EC05C-4379-49DC-8B99-679FAC8FE7DF}" name="LWD"/>
     <tableColumn id="6" xr3:uid="{A16E1008-E82E-4B63-9D13-91E4A58BEC57}" name="Billable Hours per day"/>
@@ -2772,24 +2811,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{390BA979-ED4F-4900-B38B-FEA01C46893E}">
   <dimension ref="D2:F7"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="4:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D4" s="9" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
     </row>
-    <row r="5" spans="4:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D5" t="s">
         <v>59</v>
       </c>
@@ -2797,7 +2836,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="4:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D6" t="s">
         <v>67</v>
       </c>
@@ -2805,7 +2844,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="4:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
         <v>60</v>
       </c>
@@ -2820,31 +2859,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D1F21F-45DF-4822-809D-7911E0AE1032}">
-  <dimension ref="B1:AR33"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B1:AS33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="1.453125" customWidth="1"/>
-    <col min="2" max="2" width="16.81640625" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.1796875" customWidth="1"/>
-    <col min="5" max="5" width="8.453125" customWidth="1"/>
-    <col min="6" max="6" width="7.453125" customWidth="1"/>
-    <col min="7" max="7" width="12.6328125" customWidth="1"/>
-    <col min="8" max="8" width="4.36328125" customWidth="1"/>
-    <col min="9" max="9" width="4.6328125" customWidth="1"/>
-    <col min="10" max="10" width="6.453125" customWidth="1"/>
-    <col min="11" max="11" width="9.36328125" customWidth="1"/>
-    <col min="12" max="12" width="3.6328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="37" width="6.453125" customWidth="1"/>
-    <col min="38" max="38" width="5.453125" customWidth="1"/>
+    <col min="1" max="1" width="1.5" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.1640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5" customWidth="1"/>
+    <col min="6" max="6" width="7.5" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.1640625" customWidth="1"/>
+    <col min="9" max="9" width="4.6640625" customWidth="1"/>
+    <col min="10" max="10" width="6.5" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="37" width="6.5" customWidth="1"/>
+    <col min="38" max="38" width="5.5" customWidth="1"/>
     <col min="39" max="39" width="6" customWidth="1"/>
-    <col min="40" max="40" width="6.36328125" customWidth="1"/>
-    <col min="41" max="41" width="5.81640625" customWidth="1"/>
-    <col min="42" max="42" width="5.1796875" customWidth="1"/>
-    <col min="43" max="43" width="8.81640625" customWidth="1"/>
+    <col min="40" max="40" width="6.33203125" customWidth="1"/>
+    <col min="41" max="41" width="5.83203125" customWidth="1"/>
+    <col min="42" max="42" width="5.1640625" customWidth="1"/>
+    <col min="43" max="43" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:44" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:45" x14ac:dyDescent="0.2">
       <c r="B1" s="4" t="s">
         <v>4</v>
       </c>
@@ -2855,7 +2894,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="2:44" ht="29" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:45" ht="28" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>18</v>
       </c>
@@ -2867,7 +2906,7 @@
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="4" spans="2:44" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:45" x14ac:dyDescent="0.2">
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
       <c r="L4" s="8" t="str">
@@ -2995,11 +3034,11 @@
         <v>TUE</v>
       </c>
     </row>
-    <row r="5" spans="2:44" ht="28.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="33" t="s">
+    <row r="5" spans="2:45" ht="28.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="33"/>
+      <c r="C5" s="27"/>
       <c r="E5" s="6" t="s">
         <v>70</v>
       </c>
@@ -3120,13 +3159,16 @@
       <c r="AR5" s="15" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="6" spans="2:44" ht="39" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B6" s="34">
+      <c r="AS5" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="2:45" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="28">
         <f>SUM(Table27[Final Billing Amount])</f>
-        <v>42752</v>
-      </c>
-      <c r="C6" s="35"/>
+        <v>61918</v>
+      </c>
+      <c r="C6" s="29"/>
       <c r="E6" s="20" t="s">
         <v>89</v>
       </c>
@@ -3254,12 +3296,15 @@
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B7" s="36" t="s">
+      <c r="AS6" s="39">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="7" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B7" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="36"/>
+      <c r="C7" s="30"/>
       <c r="E7" s="20" t="s">
         <v>90</v>
       </c>
@@ -3271,20 +3316,20 @@
         <f>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Name])</f>
         <v>employee2</v>
       </c>
-      <c r="H7" s="2" t="str">
+      <c r="H7" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(COUNT(Table27[[#This Row],[1]:[31]]), COUNTIF(Table27[[#This Row],[1]:[31]],"OFF"))*_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Billable Hours per day]),"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="2" t="str">
+        <v>112</v>
+      </c>
+      <c r="I7" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(Table27[[#This Row],[1]:[31]]),"")</f>
-        <v/>
+        <v>112</v>
       </c>
       <c r="J7" s="3">
         <v>30</v>
       </c>
-      <c r="K7" s="14" t="str">
+      <c r="K7" s="14">
         <f>IFERROR(Table27[[#This Row],[Actual Hours]]*Table27[[#This Row],[Rate]],"")</f>
-        <v/>
+        <v>3360</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>59</v>
@@ -3365,16 +3410,18 @@
       <c r="AP7" s="7">
         <v>8</v>
       </c>
-      <c r="AQ7" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Inactive</v>
-      </c>
-      <c r="AR7" s="17" t="e">
+      <c r="AQ7" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR7" s="17">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="2:44" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="AS7" s="39">
+        <v>1587</v>
+      </c>
+    </row>
+    <row r="8" spans="2:45" x14ac:dyDescent="0.2">
       <c r="B8" s="19"/>
       <c r="C8" s="19"/>
       <c r="E8" s="20" t="s">
@@ -3480,13 +3527,16 @@
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B9" s="37">
+      <c r="AS8" s="39">
+        <v>2440</v>
+      </c>
+    </row>
+    <row r="9" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B9" s="31">
         <f>SUM(Table27[Max Billable Hours])</f>
-        <v>1496</v>
-      </c>
-      <c r="C9" s="37"/>
+        <v>2154</v>
+      </c>
+      <c r="C9" s="31"/>
       <c r="E9" s="20" t="s">
         <v>92</v>
       </c>
@@ -3498,20 +3548,20 @@
         <f>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Name])</f>
         <v>employee4</v>
       </c>
-      <c r="H9" s="2" t="str">
+      <c r="H9" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(COUNT(Table27[[#This Row],[1]:[31]]), COUNTIF(Table27[[#This Row],[1]:[31]],"OFF"))*_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Billable Hours per day]),"")</f>
-        <v/>
-      </c>
-      <c r="I9" s="2" t="str">
+        <v>42</v>
+      </c>
+      <c r="I9" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(Table27[[#This Row],[1]:[31]]),"")</f>
-        <v/>
+        <v>42</v>
       </c>
       <c r="J9" s="3">
         <v>35</v>
       </c>
-      <c r="K9" s="14" t="str">
+      <c r="K9" s="14">
         <f>IFERROR(Table27[[#This Row],[Actual Hours]]*Table27[[#This Row],[Rate]],"")</f>
-        <v/>
+        <v>1470</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>59</v>
@@ -3606,18 +3656,20 @@
       <c r="AP9" s="7">
         <v>2</v>
       </c>
-      <c r="AQ9" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Inactive</v>
-      </c>
-      <c r="AR9" s="21" t="e">
+      <c r="AQ9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR9" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
+        <v>1</v>
+      </c>
+      <c r="AS9" s="39">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
       <c r="E10" s="20" t="s">
         <v>93</v>
       </c>
@@ -3629,20 +3681,20 @@
         <f>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Name])</f>
         <v>employee5</v>
       </c>
-      <c r="H10" s="2" t="str">
+      <c r="H10" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(COUNT(Table27[[#This Row],[1]:[31]]), COUNTIF(Table27[[#This Row],[1]:[31]],"OFF"))*_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Billable Hours per day]),"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="2" t="str">
+        <v>168</v>
+      </c>
+      <c r="I10" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(Table27[[#This Row],[1]:[31]]),"")</f>
-        <v/>
+        <v>168</v>
       </c>
       <c r="J10" s="3">
         <v>30</v>
       </c>
-      <c r="K10" s="14" t="str">
+      <c r="K10" s="14">
         <f>IFERROR(Table27[[#This Row],[Actual Hours]]*Table27[[#This Row],[Rate]],"")</f>
-        <v/>
+        <v>5040</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>59</v>
@@ -3737,18 +3789,20 @@
       <c r="AP10" s="7">
         <v>8</v>
       </c>
-      <c r="AQ10" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Inactive</v>
-      </c>
-      <c r="AR10" s="21" t="e">
+      <c r="AQ10" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR10" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
+        <v>1</v>
+      </c>
+      <c r="AS10" s="39">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
       <c r="E11" s="20" t="s">
         <v>94</v>
       </c>
@@ -3868,18 +3922,20 @@
       <c r="AP11" s="7">
         <v>8</v>
       </c>
-      <c r="AQ11" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Active</v>
+      <c r="AQ11" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="AR11" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
+      <c r="AS11" s="39">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
       <c r="E12" s="20" t="s">
         <v>95</v>
       </c>
@@ -4007,10 +4063,13 @@
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>0.76190476190476186</v>
       </c>
-    </row>
-    <row r="13" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
+      <c r="AS12" s="39">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
       <c r="E13" s="20" t="s">
         <v>96</v>
       </c>
@@ -4130,18 +4189,20 @@
       <c r="AP13" s="7">
         <v>8</v>
       </c>
-      <c r="AQ13" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Active</v>
+      <c r="AQ13" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="AR13" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>0.90476190476190477</v>
       </c>
-    </row>
-    <row r="14" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
+      <c r="AS13" s="39">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
       <c r="E14" s="20" t="s">
         <v>97</v>
       </c>
@@ -4153,20 +4214,20 @@
         <f>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Name])</f>
         <v>employee9</v>
       </c>
-      <c r="H14" s="2" t="str">
+      <c r="H14" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(COUNT(Table27[[#This Row],[1]:[31]]), COUNTIF(Table27[[#This Row],[1]:[31]],"OFF"))*_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Billable Hours per day]),"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="2" t="str">
+        <v>168</v>
+      </c>
+      <c r="I14" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(Table27[[#This Row],[1]:[31]]),"")</f>
-        <v/>
+        <v>168</v>
       </c>
       <c r="J14" s="3">
         <v>30</v>
       </c>
-      <c r="K14" s="14" t="str">
+      <c r="K14" s="14">
         <f>IFERROR(Table27[[#This Row],[Actual Hours]]*Table27[[#This Row],[Rate]],"")</f>
-        <v/>
+        <v>5040</v>
       </c>
       <c r="L14" s="7" t="s">
         <v>59</v>
@@ -4261,18 +4322,20 @@
       <c r="AP14" s="7">
         <v>8</v>
       </c>
-      <c r="AQ14" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Inactive</v>
-      </c>
-      <c r="AR14" s="21" t="e">
+      <c r="AQ14" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR14" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="15" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
+        <v>1</v>
+      </c>
+      <c r="AS14" s="39">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
       <c r="E15" s="20" t="s">
         <v>98</v>
       </c>
@@ -4392,18 +4455,20 @@
       <c r="AP15" s="7">
         <v>8</v>
       </c>
-      <c r="AQ15" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Active</v>
+      <c r="AQ15" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="AR15" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
+      <c r="AS15" s="39">
+        <v>4782</v>
+      </c>
+    </row>
+    <row r="16" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
       <c r="E16" s="20" t="s">
         <v>99</v>
       </c>
@@ -4531,10 +4596,13 @@
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>0.90476190476190477</v>
       </c>
-    </row>
-    <row r="17" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
+      <c r="AS16" s="39">
+        <v>4782</v>
+      </c>
+    </row>
+    <row r="17" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
       <c r="E17" s="20" t="s">
         <v>100</v>
       </c>
@@ -4632,18 +4700,20 @@
       <c r="AP17" s="7">
         <v>8</v>
       </c>
-      <c r="AQ17" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Active</v>
+      <c r="AQ17" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="AR17" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
+      <c r="AS17" s="39">
+        <v>4782</v>
+      </c>
+    </row>
+    <row r="18" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
       <c r="E18" s="20" t="s">
         <v>101</v>
       </c>
@@ -4771,10 +4841,13 @@
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
+      <c r="AS18" s="39">
+        <v>1389</v>
+      </c>
+    </row>
+    <row r="19" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
       <c r="E19" s="20" t="s">
         <v>102</v>
       </c>
@@ -4894,18 +4967,20 @@
       <c r="AP19" s="7">
         <v>8</v>
       </c>
-      <c r="AQ19" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Active</v>
+      <c r="AQ19" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="AR19" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
+      <c r="AS19" s="39">
+        <v>1389</v>
+      </c>
+    </row>
+    <row r="20" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
       <c r="E20" s="20" t="s">
         <v>103</v>
       </c>
@@ -4917,20 +4992,20 @@
         <f>_xlfn.XLOOKUP(Table27[[#This Row],[Emp ID]],Table1[Emp ID],Table1[Name])</f>
         <v>employee15</v>
       </c>
-      <c r="H20" s="2" t="str">
+      <c r="H20" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(COUNT(Table27[[#This Row],[1]:[31]]), COUNTIF(Table27[[#This Row],[1]:[31]],"OFF"))*_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Billable Hours per day]),"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="2" t="str">
+        <v>168</v>
+      </c>
+      <c r="I20" s="2">
         <f>IF(Table27[[#This Row],[Status]]="Active",SUM(Table27[[#This Row],[1]:[31]]),"")</f>
-        <v/>
+        <v>152</v>
       </c>
       <c r="J20" s="3">
         <v>28</v>
       </c>
-      <c r="K20" s="14" t="str">
+      <c r="K20" s="14">
         <f>IFERROR(Table27[[#This Row],[Actual Hours]]*Table27[[#This Row],[Rate]],"")</f>
-        <v/>
+        <v>4256</v>
       </c>
       <c r="L20" s="7" t="s">
         <v>59</v>
@@ -5025,18 +5100,20 @@
       <c r="AP20" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="AQ20" s="7" t="str">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP(Table27[[#This Row],[Name]],Table1[Name],Table1[Status]),"")</f>
-        <v>Inactive</v>
-      </c>
-      <c r="AR20" s="21" t="e">
+      <c r="AQ20" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR20" s="21">
         <f>Table27[[#This Row],[Actual Hours]]/Table27[[#This Row],[Max Billable Hours]]</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="21" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
+        <v>0.90476190476190477</v>
+      </c>
+      <c r="AS20" s="39">
+        <v>2670</v>
+      </c>
+    </row>
+    <row r="21" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
       <c r="G21" s="2" t="s">
@@ -5044,16 +5121,16 @@
       </c>
       <c r="H21" s="2">
         <f>SUBTOTAL(109,Table27[Max Billable Hours])</f>
-        <v>1496</v>
+        <v>2154</v>
       </c>
       <c r="I21" s="2">
         <f>SUBTOTAL(109,Table27[Actual Hours])</f>
-        <v>1424</v>
+        <v>2066</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="16">
         <f>SUBTOTAL(109,Table27[Final Billing Amount])</f>
-        <v>42752</v>
+        <v>61918</v>
       </c>
       <c r="L21" s="10">
         <f>SUBTOTAL(109,Table27[1])</f>
@@ -5182,82 +5259,83 @@
       <c r="AQ21" s="10"/>
       <c r="AR21" s="18">
         <f>Table27[[#Totals],[Actual Hours]]/Table27[[#Totals],[Max Billable Hours]]</f>
-        <v>0.95187165775401072</v>
-      </c>
-    </row>
-    <row r="23" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B23" s="38" t="s">
+        <v>0.95914577530176415</v>
+      </c>
+      <c r="AS21" s="10"/>
+    </row>
+    <row r="23" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B23" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="38"/>
-    </row>
-    <row r="24" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B24" s="32">
+      <c r="C23" s="32"/>
+    </row>
+    <row r="24" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B24" s="38">
         <f>SUM(Table27[Actual Hours])</f>
-        <v>1424</v>
-      </c>
-      <c r="C24" s="32"/>
-    </row>
-    <row r="25" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-    </row>
-    <row r="27" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B27" s="27" t="s">
+        <v>2066</v>
+      </c>
+      <c r="C24" s="38"/>
+    </row>
+    <row r="25" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+    </row>
+    <row r="27" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B27" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="27"/>
-    </row>
-    <row r="28" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B28" s="28">
+      <c r="C27" s="33"/>
+    </row>
+    <row r="28" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B28" s="34">
         <f>SUM(Table27[Actual Hours])/SUM(Table27[Max Billable Hours])</f>
-        <v>0.95187165775401072</v>
-      </c>
-      <c r="C28" s="28"/>
-    </row>
-    <row r="29" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-    </row>
-    <row r="31" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-    </row>
-    <row r="32" spans="2:44" x14ac:dyDescent="0.35">
-      <c r="B32" s="30"/>
-      <c r="C32" s="31"/>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
+        <v>0.95914577530176415</v>
+      </c>
+      <c r="C28" s="34"/>
+    </row>
+    <row r="29" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B29" s="34"/>
+      <c r="C29" s="34"/>
+    </row>
+    <row r="31" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+    </row>
+    <row r="32" spans="2:45" x14ac:dyDescent="0.2">
+      <c r="B32" s="36"/>
+      <c r="C32" s="37"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C29"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C33"/>
+    <mergeCell ref="B24:C25"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B9:C21"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C29"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C33"/>
-    <mergeCell ref="B24:C25"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="J4:AP4">
-    <cfRule type="beginsWith" dxfId="45" priority="23" operator="beginsWith" text="S">
+    <cfRule type="beginsWith" dxfId="47" priority="23" operator="beginsWith" text="S">
       <formula>LEFT(J4,LEN("S"))="S"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T6:AE6 L6:S9 L6:N19 AF6:AQ20 R7:AE7 Y7:AG8 T8:Z9 AA9:AE9 R10:AE11 L10:Q20 R12:AG12 R13:AE16 Y17:AI17 R17:Z20 AA18:AE20 L21:AQ21">
-    <cfRule type="beginsWith" dxfId="44" priority="20" operator="beginsWith" text="H">
+  <conditionalFormatting sqref="T6:AE6 L6:S9 L6:N19 R7:AE7 Y7:AG8 T8:Z9 AA9:AE9 R10:AE11 L10:Q20 R12:AG12 R13:AE16 Y17:AI17 R17:Z20 AA18:AE20 L21:AQ21 AF6:AQ20">
+    <cfRule type="beginsWith" dxfId="46" priority="20" operator="beginsWith" text="H">
       <formula>LEFT(L6,LEN("H"))="H"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="43" priority="21" operator="containsText" text="OF">
+    <cfRule type="containsText" dxfId="45" priority="21" operator="containsText" text="OF">
       <formula>NOT(ISERROR(SEARCH("OF",L6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="22" operator="containsText" text="WO">
+    <cfRule type="containsText" dxfId="44" priority="22" operator="containsText" text="WO">
       <formula>NOT(ISERROR(SEARCH("WO",L6)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5285,18 +5363,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC27336A-3765-4D13-9885-4C654CCBDEF2}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B1:H24"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.6328125" customWidth="1"/>
-    <col min="3" max="3" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>70</v>
       </c>
@@ -5319,7 +5397,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B2" s="20" t="s">
         <v>89</v>
       </c>
@@ -5339,7 +5417,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" s="20" t="s">
         <v>90</v>
       </c>
@@ -5353,13 +5431,13 @@
         <v>45525</v>
       </c>
       <c r="F3" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="H3">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B4" s="20" t="s">
         <v>91</v>
       </c>
@@ -5379,7 +5457,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
         <v>92</v>
       </c>
@@ -5393,13 +5471,13 @@
         <v>45525</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B6" s="20" t="s">
         <v>93</v>
       </c>
@@ -5419,7 +5497,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B7" s="20" t="s">
         <v>94</v>
       </c>
@@ -5439,7 +5517,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B8" s="20" t="s">
         <v>95</v>
       </c>
@@ -5459,7 +5537,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B9" s="20" t="s">
         <v>96</v>
       </c>
@@ -5479,7 +5557,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" s="20" t="s">
         <v>97</v>
       </c>
@@ -5493,13 +5571,13 @@
         <v>45525</v>
       </c>
       <c r="F10" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="H10">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B11" s="20" t="s">
         <v>98</v>
       </c>
@@ -5519,7 +5597,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" s="20" t="s">
         <v>99</v>
       </c>
@@ -5539,7 +5617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B13" s="20" t="s">
         <v>100</v>
       </c>
@@ -5559,7 +5637,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B14" s="20" t="s">
         <v>101</v>
       </c>
@@ -5579,7 +5657,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B15" s="20" t="s">
         <v>102</v>
       </c>
@@ -5599,7 +5677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
         <v>103</v>
       </c>
@@ -5613,13 +5691,13 @@
         <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="H16">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B17" s="20" t="s">
         <v>104</v>
       </c>
@@ -5639,7 +5717,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B18" s="20" t="s">
         <v>105</v>
       </c>
@@ -5659,7 +5737,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B19" s="20" t="s">
         <v>106</v>
       </c>
@@ -5673,13 +5751,13 @@
         <v>45525</v>
       </c>
       <c r="F19" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="H19">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B20" s="20" t="s">
         <v>107</v>
       </c>
@@ -5699,7 +5777,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B21" s="20" t="s">
         <v>108</v>
       </c>
@@ -5719,7 +5797,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
         <v>109</v>
       </c>
@@ -5739,7 +5817,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B23" s="20" t="s">
         <v>110</v>
       </c>
@@ -5759,18 +5837,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
       <c r="E24" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="D13:D14">
-    <cfRule type="expression" dxfId="41" priority="4">
+    <cfRule type="expression" dxfId="43" priority="4">
       <formula>LEFT(#REF!,1)="S"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18">
-    <cfRule type="expression" dxfId="40" priority="1">
+    <cfRule type="expression" dxfId="42" priority="1">
       <formula>LEFT(#REF!,1)="S"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5790,13 +5868,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D3F124-43E9-49EE-8F6D-B39FC0C3CB37}">
   <dimension ref="B1:E13"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>53</v>
       </c>
@@ -5807,7 +5885,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -5818,7 +5896,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -5829,7 +5907,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>10</v>
       </c>
@@ -5840,7 +5918,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>11</v>
       </c>
@@ -5851,7 +5929,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -5859,7 +5937,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>13</v>
       </c>
@@ -5867,7 +5945,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>7</v>
       </c>
@@ -5875,7 +5953,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>14</v>
       </c>
@@ -5883,7 +5961,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>15</v>
       </c>
@@ -5891,7 +5969,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>16</v>
       </c>
@@ -5899,7 +5977,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>17</v>
       </c>
@@ -5907,7 +5985,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>18</v>
       </c>

</xml_diff>